<commit_message>
chore: update example output files
</commit_message>
<xml_diff>
--- a/examples/output/xlsx/03-multi-sheet.xlsx
+++ b/examples/output/xlsx/03-multi-sheet.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sales Data" sheetId="1" r:id="R6f4f846cf9724587"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Rcc1a871c87cc4b01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sales Data" sheetId="1" r:id="R173791f2ccf0429e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R367feece25484d92"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>